<commit_message>
reglas: corrige 4 reglas sobre regimen/tipo contrato sin empleo real
A-045/A-046 (y sus C-282/C-283) exigian reg_cotiz_ppal_agrupado/
tipo_contr_ppal_agrupado informados a cualquiera que no fuera
Nunca_ha_cotizado. Quien nunca tuvo empleo real (solo prestacion/subsidio,
t_total_empleo=0) legitimamente no tiene "regimen/tipo de contrato con mas
tiempo cotizado" - confirmado con el usuario. Las 4 reglas ahora excluyen
ese caso (1.189 personas). 562 reglas, todas pasan salvo las esperadas.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01M3TyqKuDQEWTGv2WsG29bs
</commit_message>
<xml_diff>
--- a/tests/reglas_consistencia_v4.xlsx
+++ b/tests/reglas_consistencia_v4.xlsx
@@ -2868,12 +2868,12 @@
       </c>
       <c r="E46" s="2" t="inlineStr">
         <is>
-          <t>reg_cotiz_ppal_agrupado</t>
+          <t>causa_ult_baja</t>
         </is>
       </c>
       <c r="F46" s="2" t="inlineStr">
         <is>
-          <t>Quien no es Nunca_ha_cotizado tiene reg_cotiz_ppal_agrupado informada</t>
+          <t>Quien no es Nunca_ha_cotizado tiene causa_ult_baja informada</t>
         </is>
       </c>
       <c r="G46" s="2" t="inlineStr">
@@ -2888,7 +2888,7 @@
       </c>
       <c r="I46" s="2" t="inlineStr">
         <is>
-          <t>situacion_actual_afiliacion &lt;&gt; 'Nunca_ha_cotizado' AND reg_cotiz_ppal_agrupado IS NULL</t>
+          <t>situacion_actual_afiliacion &lt;&gt; 'Nunca_ha_cotizado' AND causa_ult_baja IS NULL</t>
         </is>
       </c>
       <c r="J46" s="2" t="inlineStr"/>
@@ -2921,12 +2921,12 @@
       </c>
       <c r="E47" s="2" t="inlineStr">
         <is>
-          <t>tipo_contr_ppal_agrupado</t>
+          <t>edad_ultimo_empleo</t>
         </is>
       </c>
       <c r="F47" s="2" t="inlineStr">
         <is>
-          <t>Quien no es Nunca_ha_cotizado tiene tipo_contr_ppal_agrupado informada</t>
+          <t>Quien no es Nunca_ha_cotizado tiene edad_ultimo_empleo informada</t>
         </is>
       </c>
       <c r="G47" s="2" t="inlineStr">
@@ -2941,7 +2941,7 @@
       </c>
       <c r="I47" s="2" t="inlineStr">
         <is>
-          <t>situacion_actual_afiliacion &lt;&gt; 'Nunca_ha_cotizado' AND tipo_contr_ppal_agrupado IS NULL</t>
+          <t>situacion_actual_afiliacion &lt;&gt; 'Nunca_ha_cotizado' AND edad_ultimo_empleo IS NULL</t>
         </is>
       </c>
       <c r="J47" s="2" t="inlineStr"/>
@@ -2974,12 +2974,12 @@
       </c>
       <c r="E48" s="2" t="inlineStr">
         <is>
-          <t>causa_ult_baja</t>
+          <t>reg_cotiz_ppal_agrupado</t>
         </is>
       </c>
       <c r="F48" s="2" t="inlineStr">
         <is>
-          <t>Quien no es Nunca_ha_cotizado tiene causa_ult_baja informada</t>
+          <t>Con empleo real, quien no es Nunca_ha_cotizado tiene reg_cotiz_ppal_agrupado informada</t>
         </is>
       </c>
       <c r="G48" s="2" t="inlineStr">
@@ -2994,7 +2994,7 @@
       </c>
       <c r="I48" s="2" t="inlineStr">
         <is>
-          <t>situacion_actual_afiliacion &lt;&gt; 'Nunca_ha_cotizado' AND causa_ult_baja IS NULL</t>
+          <t>situacion_actual_afiliacion &lt;&gt; 'Nunca_ha_cotizado' AND COALESCE(t_total_empleo, 0) &gt; 0 AND reg_cotiz_ppal_agrupado IS NULL</t>
         </is>
       </c>
       <c r="J48" s="2" t="inlineStr"/>
@@ -3027,12 +3027,12 @@
       </c>
       <c r="E49" s="2" t="inlineStr">
         <is>
-          <t>edad_ultimo_empleo</t>
+          <t>tipo_contr_ppal_agrupado</t>
         </is>
       </c>
       <c r="F49" s="2" t="inlineStr">
         <is>
-          <t>Quien no es Nunca_ha_cotizado tiene edad_ultimo_empleo informada</t>
+          <t>Con empleo real, quien no es Nunca_ha_cotizado tiene tipo_contr_ppal_agrupado informada</t>
         </is>
       </c>
       <c r="G49" s="2" t="inlineStr">
@@ -3047,7 +3047,7 @@
       </c>
       <c r="I49" s="2" t="inlineStr">
         <is>
-          <t>situacion_actual_afiliacion &lt;&gt; 'Nunca_ha_cotizado' AND edad_ultimo_empleo IS NULL</t>
+          <t>situacion_actual_afiliacion &lt;&gt; 'Nunca_ha_cotizado' AND COALESCE(t_total_empleo, 0) &gt; 0 AND tipo_contr_ppal_agrupado IS NULL</t>
         </is>
       </c>
       <c r="J49" s="2" t="inlineStr"/>
@@ -27089,7 +27089,7 @@
       </c>
       <c r="F506" s="2" t="inlineStr">
         <is>
-          <t>Sin régimen de cotización ⇒ Nunca_ha_cotizado</t>
+          <t>Sin régimen de cotización, con empleo real ⇒ Nunca_ha_cotizado</t>
         </is>
       </c>
       <c r="G506" s="2" t="inlineStr">
@@ -27104,10 +27104,14 @@
       </c>
       <c r="I506" s="2" t="inlineStr">
         <is>
-          <t>reg_cotiz_ppal_agrupado IS NULL AND situacion_actual_afiliacion &lt;&gt; 'Nunca_ha_cotizado'</t>
-        </is>
-      </c>
-      <c r="J506" s="2" t="inlineStr"/>
+          <t>reg_cotiz_ppal_agrupado IS NULL AND COALESCE(t_total_empleo, 0) &gt; 0 AND situacion_actual_afiliacion &lt;&gt; 'Nunca_ha_cotizado'</t>
+        </is>
+      </c>
+      <c r="J506" s="2" t="inlineStr">
+        <is>
+          <t>Regla corregida 2026-09-22: quien nunca tuvo empleo real (solo prestación/subsidio) no tiene régimen principal, aunque no sea Nunca_ha_cotizado (1.189 personas)</t>
+        </is>
+      </c>
       <c r="K506" s="2" t="inlineStr">
         <is>
           <t>OK</t>
@@ -27142,7 +27146,7 @@
       </c>
       <c r="F507" s="2" t="inlineStr">
         <is>
-          <t>Sin tipo de contrato principal (nulo) ⇒ Nunca_ha_cotizado</t>
+          <t>Sin tipo de contrato principal (nulo), con empleo real ⇒ Nunca_ha_cotizado</t>
         </is>
       </c>
       <c r="G507" s="2" t="inlineStr">
@@ -27157,10 +27161,14 @@
       </c>
       <c r="I507" s="2" t="inlineStr">
         <is>
-          <t>tipo_contr_ppal_agrupado IS NULL AND situacion_actual_afiliacion &lt;&gt; 'Nunca_ha_cotizado'</t>
-        </is>
-      </c>
-      <c r="J507" s="2" t="inlineStr"/>
+          <t>tipo_contr_ppal_agrupado IS NULL AND COALESCE(t_total_empleo, 0) &gt; 0 AND situacion_actual_afiliacion &lt;&gt; 'Nunca_ha_cotizado'</t>
+        </is>
+      </c>
+      <c r="J507" s="2" t="inlineStr">
+        <is>
+          <t>Regla corregida 2026-09-22: quien nunca tuvo empleo real (solo prestación/subsidio) no tiene tipo de contrato principal, aunque no sea Nunca_ha_cotizado (1.189 personas)</t>
+        </is>
+      </c>
       <c r="K507" s="2" t="inlineStr">
         <is>
           <t>OK</t>

</xml_diff>

<commit_message>
ETL: Edad_Actual_Fecha_Corte de los fallecidos se calcula a su fecha de fallecimiento
Para los 18.801 fallecidos, la edad pasa de la fecha de corte a la de fallecimiento (mes): coincide con
edad_fallecimiento y con el corte de su vida laboral (Tiempo_total_desde_inicio_VL, T_total_*). Antes salian
0,25-1,25 anyos mas viejos y 528 aparecian con mas de 100 anyos (385 por edad al fallecer). Verificado con
datos reales: fallecidos == edad_fallecimiento, no fallecidos identica, 0 negativas. Reglas: C-102 solo
para no fallecidos; C-334 pasa a "edad_actual = edad_fallecimiento en fallecidos" (debe dar 0 tras
regenerar los Parquet).

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tests/reglas_consistencia_v4.xlsx
+++ b/tests/reglas_consistencia_v4.xlsx
@@ -17198,7 +17198,7 @@
       </c>
       <c r="F315" s="2" t="inlineStr">
         <is>
-          <t>edad_actual = (1-5-2025 − nacimiento)/365,25 (±0,02)</t>
+          <t>Para no fallecidos: edad_actual = (1-5-2025 − nacimiento)/365,25 (±0,02)</t>
         </is>
       </c>
       <c r="G315" s="2" t="inlineStr">
@@ -17213,10 +17213,14 @@
       </c>
       <c r="I315" s="2" t="inlineStr">
         <is>
-          <t>ABS(edad_actual_fecha_corte - date_diff('day', fecha_nacimiento, DATE '2025-05-01') / 365.25) &gt; 0.02</t>
-        </is>
-      </c>
-      <c r="J315" s="2" t="inlineStr"/>
+          <t>ha_fallecido = 'NO' AND ABS(edad_actual_fecha_corte - date_diff('day', fecha_nacimiento, DATE '2025-05-01') / 365.25) &gt; 0.02</t>
+        </is>
+      </c>
+      <c r="J315" s="2" t="inlineStr">
+        <is>
+          <t>Ajustada 2026-09-25: los fallecidos tienen la edad calculada a su fecha de fallecimiento (ver C-334).</t>
+        </is>
+      </c>
       <c r="K315" s="2" t="inlineStr">
         <is>
           <t>OK</t>
@@ -29015,7 +29019,7 @@
       </c>
       <c r="F540" s="2" t="inlineStr">
         <is>
-          <t>La edad al fallecer es anterior a la edad a fecha de corte</t>
+          <t>Fallecidos: edad_actual_fecha_corte = edad_fallecimiento (la edad se calcula a la fecha de fallecimiento)</t>
         </is>
       </c>
       <c r="G540" s="2" t="inlineStr">
@@ -29030,12 +29034,12 @@
       </c>
       <c r="I540" s="2" t="inlineStr">
         <is>
-          <t>ha_fallecido = 'SI' AND edad_fallecimiento &gt;= edad_actual_fecha_corte</t>
+          <t>ha_fallecido = 'SI' AND ABS(edad_actual_fecha_corte - edad_fallecimiento) &gt; 0.01</t>
         </is>
       </c>
       <c r="J540" s="2" t="inlineStr">
         <is>
-          <t>Comprobación pedida por el usuario 2026-09-21</t>
+          <t>Comprobación pedida por el usuario 2026-09-21 | Reformulada 2026-09-25 (decisión del usuario): Edad_Actual_Fecha_Corte de los fallecidos se calcula a su fecha de fallecimiento. Con el Parquet anterior a esa regeneración da 18.801 incumplimientos; debe dar 0 tras regenerar.</t>
         </is>
       </c>
       <c r="K540" s="2" t="inlineStr">

</xml_diff>